<commit_message>
Record the owner's answers on the new question file; key sheet and return note updated for AI-found citations
Writer is an independent legal person who used AI to find citations; N02, N12, N15 returned; soft overlaps kept; trigger-list deviation accepted.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YEUNXbYb9LDbJLc2ziqL3n
</commit_message>
<xml_diff>
--- a/review_results/2026-10-12_new_questions_intake/Key_Review_Sheet_for_Mr_Advocate.xlsx
+++ b/review_results/2026-10-12_new_questions_intake/Key_Review_Sheet_for_Mr_Advocate.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -524,6 +524,13 @@
     </row>
     <row r="9" ht="62" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>The writer is an independent legal person who used an AI tool to find the citations and cases (owner, 12 October). Treat every citation as unverified until you have checked it exists as cited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="62" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Everything in the project is 'LLM-judged', not lawyer-validated; your review is the first lawyer's check on this key.</t>
         </is>
@@ -6027,7 +6034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6064,12 +6071,12 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Which is the primary authority for an ACCUSED's age claim: P. Yuvaprakash (2023, a victim's age) or Rishipal Singh Solanki (2021, an accused's juvenility claim)? Is Aadhaar really outside the list in s.94(2)?</t>
+          <t>The writer used an AI tool to find the citations and cases. Please check that EVERY authority named in the key exists as cited (case name, court, date, citation) and is the case the key says it is, not only what it holds. Claude found 58 of the 77 authorities named for N01 to N27 in the index; a name that is not in the index may be a real case outside the collection or a wrong or invented citation, and the index cannot tell which. Priority: Aman Preet Singh, Womb Laboratories, K. Bhaskaran, Sarabjit Kaur, Surendra Bangali, Jagtar Singh (2023), Suresh v. State of U.P. (2024), Rajinder Singh v. State of Punjab (2015), Mohan Lal v. State of Rajasthan (2015), Sorabkhan Gandhkhan Pathan, U.N. Gupta, Dilip Singh (2021), Jagdish Lakra (2026), Vishnu Kumar Gupta (2026).</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>N19</t>
+          <t>all</t>
         </is>
       </c>
       <c r="D2" s="6" t="n"/>
@@ -6080,12 +6087,12 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>The key calls Appasaheb, Abraham Ajith / Ramesh v. State of T.N., B. Jayaraj and Satya Pal Singh 'not a counted trap'. Should any of them count as a stale ruling (Supreme Court ruling overruled, modified or replaced)? Only rulings that count will be scored as stale.</t>
+          <t>Which is the primary authority for an ACCUSED's age claim: P. Yuvaprakash (2023, a victim's age) or Rishipal Singh Solanki (2021, an accused's juvenility claim)? Is Aadhaar really outside the list in s.94(2)?</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>N16, N17, N25, N27</t>
+          <t>N19</t>
         </is>
       </c>
       <c r="D3" s="6" t="n"/>
@@ -6096,12 +6103,12 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Is the answer (the IT Act s.67 charge excludes IPC s.292 for the same act) still right after the Bombay High Court Full Bench the writer mentions?</t>
+          <t>The key calls Appasaheb, Abraham Ajith / Ramesh v. State of T.N., B. Jayaraj and Satya Pal Singh 'not a counted trap'. Should any of them count as a stale ruling (Supreme Court ruling overruled, modified or replaced)? Only rulings that count will be scored as stale.</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>N14</t>
+          <t>N16, N17, N25, N27</t>
         </is>
       </c>
       <c r="D4" s="6" t="n"/>
@@ -6112,12 +6119,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>The decision in Mallikarjun Kodagali is 2:1 and Satya Pal Singh was not formally overruled. Is the position settled?</t>
+          <t>Is the answer (the IT Act s.67 charge excludes IPC s.292 for the same act) still right after the Bombay High Court Full Bench the writer mentions?</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>N27</t>
+          <t>N14</t>
         </is>
       </c>
       <c r="D5" s="6" t="n"/>
@@ -6128,12 +6135,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Manharibhai (2012) as the 'older ruling': is it right to treat it as replaced for complaints filed from 1 July 2024? Is anything else on the s.223 BNSS hearing decided by the Supreme Court before 30 June 2026?</t>
+          <t>The decision in Mallikarjun Kodagali is 2:1 and Satya Pal Singh was not formally overruled. Is the position settled?</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>N24</t>
+          <t>N27</t>
         </is>
       </c>
       <c r="D6" s="6" t="n"/>
@@ -6144,12 +6151,12 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Confirm on SCC Online or Manupatra that no Supreme Court judgment on or before 30 June 2026 deals with non-compliance with s.105 BNSS (audio-video recording of search and seizure). The writer used web searches only.</t>
+          <t>Manharibhai (2012) as the 'older ruling': is it right to treat it as replaced for complaints filed from 1 July 2024? Is anything else on the s.223 BNSS hearing decided by the Supreme Court before 30 June 2026?</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>N29</t>
+          <t>N24</t>
         </is>
       </c>
       <c r="D7" s="6" t="n"/>
@@ -6160,12 +6167,12 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>The key says no other acceptable authority exists. Please confirm, or add.</t>
+          <t>Confirm on SCC Online or Manupatra that no Supreme Court judgment on or before 30 June 2026 deals with non-compliance with s.105 BNSS (audio-video recording of search and seizure). The writer used web searches only.</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>N10, N14, N17, N24, NR2</t>
+          <t>N29</t>
         </is>
       </c>
       <c r="D8" s="6" t="n"/>
@@ -6176,12 +6183,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Is there modern Supreme Court authority on 'no resistance / earlier relationship is not consent' to add besides Mango Ram (2000) and Gurmit Singh (1996)?</t>
+          <t>The key says no other acceptable authority exists. Please confirm, or add.</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>N20</t>
+          <t>N10, N14, N17, N24, NR2</t>
         </is>
       </c>
       <c r="D9" s="6" t="n"/>
@@ -6192,12 +6199,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Please read Bilkis Yakub Rasool (8 Jan 2024) and confirm the key; the key rests on secondary reports. Confirm that the review petitions were dismissed (Sept 2024).</t>
+          <t>Is there modern Supreme Court authority on 'no resistance / earlier relationship is not consent' to add besides Mango Ram (2000) and Gurmit Singh (1996)?</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>N26</t>
+          <t>N20</t>
         </is>
       </c>
       <c r="D10" s="6" t="n"/>
@@ -6208,12 +6215,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Confirm the citation of Siddharth v. State of U.P. (the key says (2022) 1 SCC 676; the Antil judgment cites it as 2021 SCC OnLine SC 615).</t>
+          <t>Please read Bilkis Yakub Rasool (8 Jan 2024) and confirm the key; the key rests on secondary reports. Confirm that the review petitions were dismissed (Sept 2024).</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>N01</t>
+          <t>N26</t>
         </is>
       </c>
       <c r="D11" s="6" t="n"/>
@@ -6224,12 +6231,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Authorities the writer did not open (Aman Preet Singh, Ramesh Kumar, U.N. Gupta, Sarabjit Kaur, Delhi Race Club, Independent Thought ...): confirm they are right or remove them from the list of acceptable authorities. Several are in the index and can be read there (see 'Authorities in the index').</t>
+          <t>Confirm the citation of Siddharth v. State of U.P. (the key says (2022) 1 SCC 676; the Antil judgment cites it as 2021 SCC OnLine SC 615).</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>N01, N05, N11, N13, N19</t>
+          <t>N01</t>
         </is>
       </c>
       <c r="D12" s="6" t="n"/>
@@ -6240,12 +6247,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Confirm the CrPC to BNSS section mappings used in the key (170 to 190, 179 to 199, 372 to 413, 439 to 483, 438 to 482).</t>
+          <t>Authorities the writer did not open (Aman Preet Singh, Ramesh Kumar, U.N. Gupta, Sarabjit Kaur, Delhi Race Club, Independent Thought ...): confirm they are right or remove them from the list of acceptable authorities. Several are in the index and can be read there (see 'Authorities in the index').</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>N01, N05, N11, N13, N19</t>
         </is>
       </c>
       <c r="D13" s="6" t="n"/>
@@ -6256,12 +6263,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>These four questions touch the same legal ground as earlier questions (R25; ruler T15; ruler T10 and R14; ruler T08). Keep them (results will be reported with and without them) or ask the writer for replacements?</t>
+          <t>Confirm the CrPC to BNSS section mappings used in the key (170 to 190, 179 to 199, 372 to 413, 439 to 483, 438 to 482).</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>N06, N07, N13, N04</t>
+          <t>all</t>
         </is>
       </c>
       <c r="D14" s="6" t="n"/>
@@ -6272,15 +6279,31 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
+          <t>These four questions touch the same legal ground as earlier questions (R25; ruler T15; ruler T10 and R14; ruler T08). Keep them (results will be reported with and without them) or ask the writer for replacements?</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>N06, N07, N13, N04</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
           <t>Is the day of the first remand counted in the 60 days under s.187 BNSS, as Kapil Wadhawan (2023) held for the CrPC? Is the name clash with the earlier 'CBI v. Kapil Wadhawan' (2024) harmless?</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>NR1</t>
         </is>
       </c>
-      <c r="D15" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>